<commit_message>
FOC + Vel + Pos Loop (Shake)
</commit_message>
<xml_diff>
--- a/Buying List + BOM V2.xlsx
+++ b/Buying List + BOM V2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angel\Desktop\Proyectos\FOC_BLDC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0582BAA3-4B07-4ED3-8BC8-105521B64C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{723EDD2A-6D59-4893-9D6B-1E4FF317C250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="173">
   <si>
     <t>Component</t>
   </si>
@@ -544,6 +544,18 @@
   </si>
   <si>
     <t>0603 - 600R, 100Mhz</t>
+  </si>
+  <si>
+    <t>Soldering Air Station</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>Main Asturion PCB + Smaller Stencil</t>
+  </si>
+  <si>
+    <t>2nd Component Order</t>
   </si>
 </sst>
 </file>
@@ -1461,8 +1473,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{57113999-89B8-4DCA-AAEB-0496B38A0B13}" name="Table1" displayName="Table1" ref="A1:K30" totalsRowCount="1" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25">
-  <autoFilter ref="A1:K29" xr:uid="{57113999-89B8-4DCA-AAEB-0496B38A0B13}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{57113999-89B8-4DCA-AAEB-0496B38A0B13}" name="Table1" displayName="Table1" ref="A1:K34" totalsRowCount="1" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25">
+  <autoFilter ref="A1:K33" xr:uid="{57113999-89B8-4DCA-AAEB-0496B38A0B13}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{C01A5BB4-2776-4DA4-B397-20536FB6B151}" name="Component" dataDxfId="24" totalsRowDxfId="23"/>
     <tableColumn id="2" xr3:uid="{D16A6BB5-FB54-4A08-8F36-6F894F571CA2}" name="Supplier" dataDxfId="22" totalsRowDxfId="21"/>
@@ -1773,7 +1785,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="58.109375" customWidth="1"/>
@@ -1887,7 +1899,7 @@
         <v>25</v>
       </c>
       <c r="I3" s="25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J3" s="26">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
@@ -2093,7 +2105,7 @@
         <v>25</v>
       </c>
       <c r="I9" s="25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J9" s="26">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
@@ -2226,10 +2238,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I13" s="25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J13" s="26">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
@@ -2260,10 +2272,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I14" s="25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J14" s="14">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
@@ -2621,7 +2633,7 @@
         <v>25</v>
       </c>
       <c r="I25" s="25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J25" s="26">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
@@ -2635,10 +2647,16 @@
       <c r="C26" s="13"/>
       <c r="D26" s="11"/>
       <c r="E26" s="11"/>
-      <c r="F26" s="29"/>
+      <c r="F26" s="29">
+        <v>0</v>
+      </c>
       <c r="G26" s="13"/>
-      <c r="H26" s="23"/>
-      <c r="I26" s="25"/>
+      <c r="H26" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="I26" s="25" t="s">
+        <v>25</v>
+      </c>
       <c r="J26" s="26">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
         <v>0</v>
@@ -2647,16 +2665,26 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B27" s="11"/>
+        <v>171</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>40</v>
+      </c>
       <c r="C27" s="13"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
+      <c r="D27" s="11">
+        <v>1</v>
+      </c>
+      <c r="E27" s="11">
+        <v>1</v>
+      </c>
       <c r="F27" s="29"/>
       <c r="G27" s="13"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="25"/>
+      <c r="H27" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="I27" s="25" t="s">
+        <v>26</v>
+      </c>
       <c r="J27" s="26">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
         <v>0</v>
@@ -2665,16 +2693,26 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="B28" s="11"/>
+        <v>172</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>19</v>
+      </c>
       <c r="C28" s="13"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
+      <c r="D28" s="11">
+        <v>1</v>
+      </c>
+      <c r="E28" s="11">
+        <v>1</v>
+      </c>
       <c r="F28" s="29"/>
       <c r="G28" s="13"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="25"/>
+      <c r="H28" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="I28" s="25" t="s">
+        <v>26</v>
+      </c>
       <c r="J28" s="26">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
         <v>0</v>
@@ -2682,18 +2720,35 @@
       <c r="K28" s="11"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A29" s="12"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="29"/>
+      <c r="A29" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="C29" s="13">
+        <f>50*1.15</f>
+        <v>57.499999999999993</v>
+      </c>
+      <c r="D29" s="11">
+        <v>1</v>
+      </c>
+      <c r="E29" s="11">
+        <v>1</v>
+      </c>
+      <c r="F29" s="29">
+        <v>0</v>
+      </c>
       <c r="G29" s="13"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="25"/>
-      <c r="J29" s="14">
+      <c r="H29" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="I29" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="J29" s="26">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
-        <v>0</v>
+        <v>57.499999999999993</v>
       </c>
       <c r="K29" s="11"/>
     </row>
@@ -2707,19 +2762,87 @@
       <c r="G30" s="13"/>
       <c r="H30" s="23"/>
       <c r="I30" s="25"/>
-      <c r="J30" s="14">
+      <c r="J30" s="26">
+        <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
+        <v>0</v>
+      </c>
+      <c r="K30" s="11"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" s="11"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="26">
+        <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
+        <v>0</v>
+      </c>
+      <c r="K31" s="11"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="11"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="26">
+        <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
+        <v>0</v>
+      </c>
+      <c r="K32" s="11"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="12"/>
+      <c r="B33" s="11"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="13"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="14">
+        <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Total Quantity 6 + 2]]+Table1[[#This Row],[Shipping Costs]]</f>
+        <v>0</v>
+      </c>
+      <c r="K33" s="11"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="12"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="13"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="14">
         <f>SUM(Table1[Total])</f>
-        <v>230.66</v>
-      </c>
-      <c r="K30" s="11"/>
+        <v>288.15999999999997</v>
+      </c>
+      <c r="K34" s="11"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F30">
+  <conditionalFormatting sqref="F2:F34">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:I30">
+  <conditionalFormatting sqref="H2:I34">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -2859,12 +2982,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>28</v>
       </c>
-      <c r="H4">
-        <v>40</v>
-      </c>
       <c r="I4">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="L4" s="33"/>
       <c r="M4" s="33"/>
@@ -2889,12 +3009,10 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H5" s="38">
-        <v>50</v>
-      </c>
+      <c r="H5" s="38"/>
       <c r="I5" s="39">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L5" s="33" t="s">
         <v>58</v>
@@ -2921,12 +3039,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H6">
-        <v>50</v>
-      </c>
       <c r="I6" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -2979,12 +3094,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H8">
-        <v>50</v>
-      </c>
       <c r="I8" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
@@ -3005,12 +3117,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>14</v>
       </c>
-      <c r="H9">
-        <v>40</v>
-      </c>
       <c r="I9" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -3031,12 +3140,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>63</v>
       </c>
-      <c r="H10">
-        <v>150</v>
-      </c>
       <c r="I10" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
@@ -3058,7 +3164,7 @@
         <v>14</v>
       </c>
       <c r="H11">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="I11" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
@@ -3083,12 +3189,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>28</v>
       </c>
-      <c r="H12">
-        <v>70</v>
-      </c>
       <c r="I12" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -3109,12 +3212,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H13">
-        <v>30</v>
-      </c>
       <c r="I13" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
@@ -3135,12 +3235,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>14</v>
       </c>
-      <c r="H14">
-        <v>50</v>
-      </c>
       <c r="I14" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
@@ -3187,12 +3284,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>14</v>
       </c>
-      <c r="H16">
-        <v>25</v>
-      </c>
       <c r="I16" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
@@ -3213,12 +3307,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H17">
-        <v>40</v>
-      </c>
       <c r="I17" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
@@ -3239,12 +3330,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>14</v>
       </c>
-      <c r="H18">
-        <v>50</v>
-      </c>
       <c r="I18" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
@@ -3268,12 +3356,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>14</v>
       </c>
-      <c r="H19">
-        <v>35</v>
-      </c>
       <c r="I19" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
@@ -3294,12 +3379,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H20">
-        <v>50</v>
-      </c>
       <c r="I20" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -3324,12 +3406,10 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H21" s="46">
-        <v>20</v>
-      </c>
+      <c r="H21" s="46"/>
       <c r="I21" s="47">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
@@ -3378,12 +3458,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>14</v>
       </c>
-      <c r="H23">
-        <v>60</v>
-      </c>
       <c r="I23" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
@@ -3430,12 +3507,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H25">
-        <v>30</v>
-      </c>
       <c r="I25" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
@@ -3456,12 +3530,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>14</v>
       </c>
-      <c r="H26">
-        <v>60</v>
-      </c>
       <c r="I26" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
@@ -3488,12 +3559,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>28</v>
       </c>
-      <c r="H27">
-        <v>50</v>
-      </c>
       <c r="I27" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>28</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
@@ -3514,12 +3582,9 @@
         <f>Table2[[#This Row],[Quantity]]*M5</f>
         <v>12</v>
       </c>
-      <c r="H28">
-        <v>35</v>
-      </c>
       <c r="I28" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
@@ -3540,12 +3605,9 @@
         <f>Table2[[#This Row],[Quantity]]*($M$3-M6)</f>
         <v>42</v>
       </c>
-      <c r="H29">
-        <v>76</v>
-      </c>
       <c r="I29" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
@@ -3598,12 +3660,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>14</v>
       </c>
-      <c r="H31">
-        <v>50</v>
-      </c>
       <c r="I31" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
@@ -3624,12 +3683,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H32">
-        <v>20</v>
-      </c>
       <c r="I32" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
@@ -3656,12 +3712,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>28</v>
       </c>
-      <c r="H33">
-        <v>70</v>
-      </c>
       <c r="I33" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="J33" t="s">
         <v>160</v>
@@ -3688,12 +3741,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H34">
-        <v>50</v>
-      </c>
       <c r="I34" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
@@ -3714,12 +3764,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H35">
-        <v>20</v>
-      </c>
       <c r="I35" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
@@ -3740,12 +3787,9 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H36">
-        <v>35</v>
-      </c>
       <c r="I36" s="41">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -3768,12 +3812,10 @@
         <f>Table2[[#This Row],[Quantity]]*$M$3</f>
         <v>7</v>
       </c>
-      <c r="H37" s="46">
-        <v>30</v>
-      </c>
+      <c r="H37" s="46"/>
       <c r="I37" s="47">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
@@ -4207,11 +4249,11 @@
         <v>7</v>
       </c>
       <c r="H52">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I52">
         <f>IF(Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]]&lt;=0,0,Table2[[#This Row],[Total]]-Table2[[#This Row],[Personal Stock]])</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>